<commit_message>
refactor: Localize excel logger sheets, columns to Korean and format timestamp to date only
</commit_message>
<xml_diff>
--- a/stock_portfolio_log.xlsx
+++ b/stock_portfolio_log.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Holdings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자산요약" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보유종목" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,7 +138,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Portfolio Total Asset (KRW) Trend</a:t>
+              <a:t>포트폴리오 총평가자산(원) 추이</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -152,7 +152,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Summary'!B1</f>
+              <f>'자산요약'!B1</f>
             </strRef>
           </tx>
           <spPr>
@@ -170,12 +170,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$4</f>
+              <f>'자산요약'!$A$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$B$2:$B$4</f>
+              <f>'자산요약'!$B$2</f>
             </numRef>
           </val>
         </ser>
@@ -197,7 +197,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Timestamp</a:t>
+                  <a:t>날짜</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -224,7 +224,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Total Asset (KRW)</a:t>
+                  <a:t>총평가자산 (KRW)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -257,7 +257,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Portfolio Profit Percentage (%) Trend</a:t>
+              <a:t>포트폴리오 수익률(%) 추이</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -271,7 +271,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Summary'!F1</f>
+              <f>'자산요약'!F1</f>
             </strRef>
           </tx>
           <spPr>
@@ -289,12 +289,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$4</f>
+              <f>'자산요약'!$A$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$F$2:$F$4</f>
+              <f>'자산요약'!$F$2</f>
             </numRef>
           </val>
         </ser>
@@ -316,7 +316,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Timestamp</a:t>
+                  <a:t>날짜</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -343,7 +343,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Profit Pct (%)</a:t>
+                  <a:t>수익률 (%)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -701,132 +701,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>날짜</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Total_Asset_KRW</t>
+          <t>총평가자산(원)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Cash_USD</t>
+          <t>예수금($)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Eval_USD</t>
+          <t>주식평가금액($)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Profit_USD</t>
+          <t>평가손익($)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Profit_Pct</t>
+          <t>수익률(%)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>사이클</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Tranche</t>
+          <t>회차</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-18 21:00:36</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>28836747</v>
+        <v>28839720</v>
       </c>
       <c r="C2" t="n">
-        <v>20376.45</v>
+        <v>20378.55</v>
       </c>
       <c r="D2" t="n">
-        <v>652.54</v>
+        <v>654.64</v>
       </c>
       <c r="E2" t="n">
-        <v>-61.35</v>
+        <v>-59.25</v>
       </c>
       <c r="F2" t="n">
-        <v>-8.59</v>
+        <v>-8.289999999999999</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-18 21:00:51</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>28837201</v>
-      </c>
-      <c r="C3" t="n">
-        <v>20376.77</v>
-      </c>
-      <c r="D3" t="n">
-        <v>652.86</v>
-      </c>
-      <c r="E3" t="n">
-        <v>-61.03</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-8.539999999999999</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-18 21:02:04</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>28837851</v>
-      </c>
-      <c r="C4" t="n">
-        <v>20377.23</v>
-      </c>
-      <c r="D4" t="n">
-        <v>653.3200000000001</v>
-      </c>
-      <c r="E4" t="n">
-        <v>-60.57</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-8.48</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -842,50 +786,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>날짜</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Ticker</t>
+          <t>티커</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>종목명</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Qty</t>
+          <t>보유수량</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>AvgPrice</t>
+          <t>평균단가($)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>CurPrice</t>
+          <t>현재가($)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>ProfitPct</t>
+          <t>수익률(%)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-18 21:00:36</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -905,16 +849,16 @@
         <v>153.2</v>
       </c>
       <c r="F2" t="n">
-        <v>135.57</v>
+        <v>136.2</v>
       </c>
       <c r="G2" t="n">
-        <v>-11.5</v>
+        <v>-11.09</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-18 21:00:36</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -943,7 +887,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-18 21:00:36</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -963,184 +907,10 @@
         <v>76.51000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>73.8</v>
+        <v>73.87</v>
       </c>
       <c r="G4" t="n">
-        <v>-3.55</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-18 21:00:51</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>SOXL</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>디렉시온 반도체 3배 ETF</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" t="n">
-        <v>153.2</v>
-      </c>
-      <c r="F5" t="n">
-        <v>135.64</v>
-      </c>
-      <c r="G5" t="n">
-        <v>-11.45</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-18 21:00:51</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>IQQ</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>ISHARES NASDAQ 100 ETF</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="n">
-        <v>24.74</v>
-      </c>
-      <c r="F6" t="n">
-        <v>24.43</v>
-      </c>
-      <c r="G6" t="n">
-        <v>-1.25</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-18 21:00:51</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>TQQQ</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>프로셰어즈 QQQ 3배 ETF</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" t="n">
-        <v>76.51000000000001</v>
-      </c>
-      <c r="F7" t="n">
-        <v>73.83</v>
-      </c>
-      <c r="G7" t="n">
-        <v>-3.51</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-08-18 21:02:04</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>SOXL</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>디렉시온 반도체 3배 ETF</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E8" t="n">
-        <v>153.2</v>
-      </c>
-      <c r="F8" t="n">
-        <v>135.8</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-11.35</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-08-18 21:02:04</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>IQQ</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>ISHARES NASDAQ 100 ETF</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="n">
-        <v>24.74</v>
-      </c>
-      <c r="F9" t="n">
-        <v>24.43</v>
-      </c>
-      <c r="G9" t="n">
-        <v>-1.25</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-08-18 21:02:04</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>TQQQ</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>프로셰어즈 QQQ 3배 ETF</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E10" t="n">
-        <v>76.51000000000001</v>
-      </c>
-      <c r="F10" t="n">
-        <v>73.83</v>
-      </c>
-      <c r="G10" t="n">
-        <v>-3.51</v>
+        <v>-3.45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add target-profit take-profit sell order generation in order_executor.py
</commit_message>
<xml_diff>
--- a/stock_portfolio_log.xlsx
+++ b/stock_portfolio_log.xlsx
@@ -170,12 +170,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'자산요약'!$A$2</f>
+              <f>'자산요약'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'자산요약'!$B$2</f>
+              <f>'자산요약'!$B$2:$B$3</f>
             </numRef>
           </val>
         </ser>
@@ -289,12 +289,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'자산요약'!$A$2</f>
+              <f>'자산요약'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'자산요약'!$F$2</f>
+              <f>'자산요약'!$F$2:$F$3</f>
             </numRef>
           </val>
         </ser>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -745,6 +745,16 @@
           <t>회차</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>SOXL(사이클/회차)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>TQQQ(사이클/회차)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -772,6 +782,38 @@
       </c>
       <c r="H2" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>28844413</v>
+      </c>
+      <c r="C3" t="n">
+        <v>20381.86</v>
+      </c>
+      <c r="D3" t="n">
+        <v>657.95</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-55.94</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-7.83</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>#1 / 1회차</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>#1 / 1회차</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -786,7 +828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -911,6 +953,93 @@
       </c>
       <c r="G4" t="n">
         <v>-3.45</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>디렉시온 반도체 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>153.2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>137.1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-10.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>IQQ</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ISHARES NASDAQ 100 ETF</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="F6" t="n">
+        <v>24.45</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-1.17</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>프로셰어즈 QQQ 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="n">
+        <v>76.51000000000001</v>
+      </c>
+      <c r="F7" t="n">
+        <v>74.06</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-3.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Calculate total_asset_usd correctly from cash and eval amount
</commit_message>
<xml_diff>
--- a/stock_portfolio_log.xlsx
+++ b/stock_portfolio_log.xlsx
@@ -170,12 +170,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'자산요약'!$A$2:$A$3</f>
+              <f>'자산요약'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'자산요약'!$B$2:$B$3</f>
+              <f>'자산요약'!$B$2:$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -289,12 +289,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'자산요약'!$A$2:$A$3</f>
+              <f>'자산요약'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'자산요약'!$F$2:$F$3</f>
+              <f>'자산요약'!$F$2:$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -811,6 +811,70 @@
         </is>
       </c>
       <c r="J3" t="inlineStr">
+        <is>
+          <t>#1 / 1회차</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>28829345</v>
+      </c>
+      <c r="C4" t="n">
+        <v>20371.22</v>
+      </c>
+      <c r="D4" t="n">
+        <v>647.3099999999999</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-66.58</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-9.32</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>#1 / 1회차</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>#1 / 1회차</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>28828798</v>
+      </c>
+      <c r="C5" t="n">
+        <v>20370.83</v>
+      </c>
+      <c r="D5" t="n">
+        <v>646.92</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-66.97</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-9.380000000000001</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>#1 / 1회차</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>#1 / 1회차</t>
         </is>
@@ -828,7 +892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1042,6 +1106,180 @@
         <v>-3.2</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>디렉시온 반도체 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>153.2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>134.33</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-12.31</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>IQQ</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ISHARES NASDAQ 100 ETF</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="F9" t="n">
+        <v>24.39</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-1.41</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>프로셰어즈 QQQ 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>76.51000000000001</v>
+      </c>
+      <c r="F10" t="n">
+        <v>73.31</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-4.19</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>디렉시온 반도체 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="n">
+        <v>153.2</v>
+      </c>
+      <c r="F11" t="n">
+        <v>134.21</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-12.39</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>IQQ</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ISHARES NASDAQ 100 ETF</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="F12" t="n">
+        <v>24.35</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-1.57</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>프로셰어즈 QQQ 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>76.51000000000001</v>
+      </c>
+      <c r="F13" t="n">
+        <v>73.31</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-4.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Upgrade quant engine and excel logger to official Lao-er Infinite Buy Method V4.0 rules
</commit_message>
<xml_diff>
--- a/stock_portfolio_log.xlsx
+++ b/stock_portfolio_log.xlsx
@@ -170,12 +170,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'자산요약'!$A$2:$A$5</f>
+              <f>'자산요약'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'자산요약'!$B$2:$B$5</f>
+              <f>'자산요약'!$B$2:$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -289,12 +289,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'자산요약'!$A$2:$A$5</f>
+              <f>'자산요약'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'자산요약'!$F$2:$F$5</f>
+              <f>'자산요약'!$F$2:$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -755,6 +755,16 @@
           <t>TQQQ(사이클/회차)</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>SOXL(사이클/T)</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>TQQQ(사이클/T)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -877,6 +887,38 @@
       <c r="J5" t="inlineStr">
         <is>
           <t>#1 / 1회차</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>28833294</v>
+      </c>
+      <c r="C6" t="n">
+        <v>20374.01</v>
+      </c>
+      <c r="D6" t="n">
+        <v>650.1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-63.79</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-8.93</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>#1 / T=0.0</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>#1 / T=0.0</t>
         </is>
       </c>
     </row>
@@ -892,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1280,6 +1322,93 @@
         <v>-4.19</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>디렉시온 반도체 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" t="n">
+        <v>153.2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>134.86</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-11.97</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>IQQ</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ISHARES NASDAQ 100 ETF</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="F15" t="n">
+        <v>24.39</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-1.41</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>프로셰어즈 QQQ 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="n">
+        <v>76.51000000000001</v>
+      </c>
+      <c r="F16" t="n">
+        <v>73.70999999999999</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-3.66</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Integrate V4.0 live order execution into main.py for full-auto GitHub Actions workflow
</commit_message>
<xml_diff>
--- a/stock_portfolio_log.xlsx
+++ b/stock_portfolio_log.xlsx
@@ -170,12 +170,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'자산요약'!$A$2:$A$6</f>
+              <f>'자산요약'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'자산요약'!$B$2:$B$6</f>
+              <f>'자산요약'!$B$2:$B$8</f>
             </numRef>
           </val>
         </ser>
@@ -289,12 +289,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'자산요약'!$A$2:$A$6</f>
+              <f>'자산요약'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'자산요약'!$F$2:$F$6</f>
+              <f>'자산요약'!$F$2:$F$8</f>
             </numRef>
           </val>
         </ser>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -919,6 +919,70 @@
       <c r="L6" t="inlineStr">
         <is>
           <t>#1 / T=0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>28814899</v>
+      </c>
+      <c r="C7" t="n">
+        <v>20360.99</v>
+      </c>
+      <c r="D7" t="n">
+        <v>637.08</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-76.81</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-10.75</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>#1 / T=0.0</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>#1 / T=0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>28810829</v>
+      </c>
+      <c r="C8" t="n">
+        <v>20358.13</v>
+      </c>
+      <c r="D8" t="n">
+        <v>634.22</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-79.67</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-11.15</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>#1 / T=1.0</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>#1 / T=1.0</t>
         </is>
       </c>
     </row>
@@ -934,7 +998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1409,6 +1473,180 @@
         <v>-3.66</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>디렉시온 반도체 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="n">
+        <v>153.2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>131.13</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-14.4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>IQQ</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ISHARES NASDAQ 100 ETF</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="F18" t="n">
+        <v>24.34</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-1.61</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>프로셰어즈 QQQ 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="n">
+        <v>76.51000000000001</v>
+      </c>
+      <c r="F19" t="n">
+        <v>73.11</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-4.44</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>디렉시온 반도체 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="n">
+        <v>153.2</v>
+      </c>
+      <c r="F20" t="n">
+        <v>130.29</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-14.95</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>IQQ</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ISHARES NASDAQ 100 ETF</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="F21" t="n">
+        <v>24.32</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-1.69</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>프로셰어즈 QQQ 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" t="n">
+        <v>76.51000000000001</v>
+      </c>
+      <c r="F22" t="n">
+        <v>73.01000000000001</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-4.58</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
security: Remove hardcoded plaintext API keys and Telegram tokens from config.py
</commit_message>
<xml_diff>
--- a/stock_portfolio_log.xlsx
+++ b/stock_portfolio_log.xlsx
@@ -170,12 +170,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'자산요약'!$A$2:$A$8</f>
+              <f>'자산요약'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'자산요약'!$B$2:$B$8</f>
+              <f>'자산요약'!$B$2:$B$9</f>
             </numRef>
           </val>
         </ser>
@@ -289,12 +289,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'자산요약'!$A$2:$A$8</f>
+              <f>'자산요약'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'자산요약'!$F$2:$F$8</f>
+              <f>'자산요약'!$F$2:$F$9</f>
             </numRef>
           </val>
         </ser>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -981,6 +981,38 @@
         </is>
       </c>
       <c r="L8" t="inlineStr">
+        <is>
+          <t>#1 / T=1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>28808160</v>
+      </c>
+      <c r="C9" t="n">
+        <v>20356.25</v>
+      </c>
+      <c r="D9" t="n">
+        <v>632.34</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-81.55</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-11.42</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>#1 / T=1.0</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>#1 / T=1.0</t>
         </is>
@@ -998,7 +1030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1647,6 +1679,93 @@
         <v>-4.58</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>디렉시온 반도체 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>153.2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>129.73</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-15.31</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>IQQ</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ISHARES NASDAQ 100 ETF</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="F24" t="n">
+        <v>24.33</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-1.65</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>프로셰어즈 QQQ 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" t="n">
+        <v>76.51000000000001</v>
+      </c>
+      <c r="F25" t="n">
+        <v>72.94</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-4.67</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add V4.0 quantity multiplier (double/half tranche) and config fixes
</commit_message>
<xml_diff>
--- a/stock_portfolio_log.xlsx
+++ b/stock_portfolio_log.xlsx
@@ -170,12 +170,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'자산요약'!$A$2:$A$9</f>
+              <f>'자산요약'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'자산요약'!$B$2:$B$9</f>
+              <f>'자산요약'!$B$2:$B$12</f>
             </numRef>
           </val>
         </ser>
@@ -289,12 +289,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'자산요약'!$A$2:$A$9</f>
+              <f>'자산요약'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'자산요약'!$F$2:$F$9</f>
+              <f>'자산요약'!$F$2:$F$12</f>
             </numRef>
           </val>
         </ser>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1013,6 +1013,102 @@
         </is>
       </c>
       <c r="L9" t="inlineStr">
+        <is>
+          <t>#1 / T=1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>28811953</v>
+      </c>
+      <c r="C10" t="n">
+        <v>20358.92</v>
+      </c>
+      <c r="D10" t="n">
+        <v>635.01</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-78.88</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-11.04</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>#1 / T=1.0</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>#1 / T=1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>28810976</v>
+      </c>
+      <c r="C11" t="n">
+        <v>20358.23</v>
+      </c>
+      <c r="D11" t="n">
+        <v>634.3200000000001</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-79.56999999999999</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-11.14</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>#1 / T=1.0</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>#1 / T=1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>28809116</v>
+      </c>
+      <c r="C12" t="n">
+        <v>20356.92</v>
+      </c>
+      <c r="D12" t="n">
+        <v>633.01</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-80.88</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-11.32</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>#1 / T=1.0</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>#1 / T=1.0</t>
         </is>
@@ -1030,7 +1126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1766,6 +1862,267 @@
         <v>-4.67</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>디렉시온 반도체 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>3</v>
+      </c>
+      <c r="E26" t="n">
+        <v>153.2</v>
+      </c>
+      <c r="F26" t="n">
+        <v>130.51</v>
+      </c>
+      <c r="G26" t="n">
+        <v>-14.8</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>IQQ</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ISHARES NASDAQ 100 ETF</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="F27" t="n">
+        <v>24.32</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-1.69</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>프로셰어즈 QQQ 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" t="n">
+        <v>76.51000000000001</v>
+      </c>
+      <c r="F28" t="n">
+        <v>73.05</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-4.53</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>디렉시온 반도체 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" t="n">
+        <v>153.2</v>
+      </c>
+      <c r="F29" t="n">
+        <v>130.33</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-14.92</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>IQQ</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ISHARES NASDAQ 100 ETF</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="F30" t="n">
+        <v>24.33</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-1.65</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>프로셰어즈 QQQ 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" t="n">
+        <v>76.51000000000001</v>
+      </c>
+      <c r="F31" t="n">
+        <v>72.98999999999999</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-4.6</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>디렉시온 반도체 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" t="n">
+        <v>153.2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>129.79</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-15.28</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>IQQ</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ISHARES NASDAQ 100 ETF</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="F33" t="n">
+        <v>24.34</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-1.61</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>프로셰어즈 QQQ 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" t="n">
+        <v>76.51000000000001</v>
+      </c>
+      <c r="F34" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-4.46</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Add idempotency check to prevent duplicate stock orders and configure GHA concurrency
</commit_message>
<xml_diff>
--- a/stock_portfolio_log.xlsx
+++ b/stock_portfolio_log.xlsx
@@ -170,12 +170,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'자산요약'!$A$2:$A$12</f>
+              <f>'자산요약'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'자산요약'!$B$2:$B$12</f>
+              <f>'자산요약'!$B$2:$B$13</f>
             </numRef>
           </val>
         </ser>
@@ -289,12 +289,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'자산요약'!$A$2:$A$12</f>
+              <f>'자산요약'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'자산요약'!$F$2:$F$12</f>
+              <f>'자산요약'!$F$2:$F$13</f>
             </numRef>
           </val>
         </ser>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1109,6 +1109,38 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>#1 / T=1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>28773607</v>
+      </c>
+      <c r="C13" t="n">
+        <v>20392.35</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2112.05</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-44.34</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-2.05</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>#1 / T=1.0</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>#1 / T=1.0</t>
         </is>
@@ -1126,7 +1158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2123,6 +2155,122 @@
         <v>-4.46</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>디렉시온 반도체 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>8</v>
+      </c>
+      <c r="E35" t="n">
+        <v>137.7</v>
+      </c>
+      <c r="F35" t="n">
+        <v>133.05</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-3.38</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>IQQ</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ISHARES NASDAQ 100 ETF</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="F36" t="n">
+        <v>24.37</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-1.49</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>QLD</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>프로셰어즈 QQQ 2배 ETF</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>4</v>
+      </c>
+      <c r="E37" t="n">
+        <v>91.2</v>
+      </c>
+      <c r="F37" t="n">
+        <v>91.20999999999999</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>프로셰어즈 QQQ 3배 ETF</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>9</v>
+      </c>
+      <c r="E38" t="n">
+        <v>73.91</v>
+      </c>
+      <c r="F38" t="n">
+        <v>73.16</v>
+      </c>
+      <c r="G38" t="n">
+        <v>-1.01</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>